<commit_message>
added new function for reading the secret name
</commit_message>
<xml_diff>
--- a/gcp_training/sample_data.xlsx
+++ b/gcp_training/sample_data.xlsx
@@ -1,15 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Windows 10\Desktop\MyData\gcp_training\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="90" windowWidth="13395" windowHeight="3405"/>
+    <workbookView xWindow="0" yWindow="90" windowWidth="13400" windowHeight="3410"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
@@ -90,9 +93,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -147,7 +150,7 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -177,6 +180,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -225,7 +231,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -260,7 +266,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -470,16 +476,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -496,7 +502,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -513,7 +519,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -530,7 +536,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -547,7 +553,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -564,7 +570,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -581,7 +587,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -598,7 +604,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
@@ -615,7 +621,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -632,7 +638,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -649,7 +655,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
@@ -666,7 +672,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
@@ -683,7 +689,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -700,7 +706,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>5</v>
       </c>
@@ -717,7 +723,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>5</v>
       </c>
@@ -734,7 +740,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>5</v>
       </c>
@@ -751,7 +757,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>5</v>
       </c>
@@ -768,7 +774,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
         <v>5</v>
       </c>
@@ -785,7 +791,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
         <v>7</v>
       </c>
@@ -802,7 +808,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
         <v>5</v>
       </c>
@@ -819,7 +825,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
         <v>7</v>
       </c>
@@ -836,7 +842,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
         <v>5</v>
       </c>
@@ -853,7 +859,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
         <v>7</v>
       </c>
@@ -873,22 +879,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>